<commit_message>
Zielgruppe 2: Müller - Die lila Logistik entfernt
Kontraktlogistiker-Liste umfasst damit 30 Einträge.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KugR1U5dxR4p4yhkLqU2yh
</commit_message>
<xml_diff>
--- a/adresslisten/Zielgruppe_2_Kontraktlogistiker_WMS.xlsx
+++ b/adresslisten/Zielgruppe_2_Kontraktlogistiker_WMS.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Kontraktlogistiker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Kontraktlogistiker'!$A$1:$C$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Kontraktlogistiker'!$A$1:$C$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -539,464 +539,447 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Müller – Die lila Logistik SE</t>
+          <t>Hammer GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>https://www.lila-logistik.com</t>
+          <t>https://www.hammer-ac.de</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>+49 7143 810-0</t>
+          <t>+49 241 9665-0</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Hammer GmbH &amp; Co. KG</t>
+          <t>Rieck Holding GmbH &amp; Co. KG (Rieck Logistik-Gruppe)</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>https://www.hammer-ac.de</t>
+          <t>https://www.rieck-logistik.de</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>+49 241 9665-0</t>
+          <t>+49 33701 339-0</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Rieck Holding GmbH &amp; Co. KG (Rieck Logistik-Gruppe)</t>
+          <t>Honold Logistik &amp; Immobilien Gruppe GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>https://www.rieck-logistik.de</t>
+          <t>https://www.honold.net</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>+49 33701 339-0</t>
+          <t>+49 731 9754-0</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Honold Logistik &amp; Immobilien Gruppe GmbH &amp; Co. KG</t>
+          <t>Friedrich Zufall GmbH &amp; Co. KG (ZUFALL logistics group)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>https://www.honold.net</t>
+          <t>https://www.zufall.de</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>+49 731 9754-0</t>
+          <t>+49 551 607-0</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Friedrich Zufall GmbH &amp; Co. KG (ZUFALL logistics group)</t>
+          <t>Schäflein AG</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>https://www.zufall.de</t>
+          <t>https://www.schaeflein.de</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>+49 551 607-0</t>
+          <t>+49 9723 9069-0</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Schäflein AG</t>
+          <t>Noerpel SE</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>https://www.schaeflein.de</t>
+          <t>https://www.noerpel.de</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>+49 9723 9069-0</t>
+          <t>+49 731 4005-0</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Noerpel SE</t>
+          <t>TST GmbH (Trans Service Team)</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>https://www.noerpel.de</t>
+          <t>https://www.trans-service-team.com</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>+49 731 4005-0</t>
+          <t>+49 6242 91508-0</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TST GmbH (Trans Service Team)</t>
+          <t>Rüdinger Spedition GmbH</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>https://www.trans-service-team.com</t>
+          <t>https://www.spedition-ruedinger.de</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>+49 6242 91508-0</t>
+          <t>+49 6294 908-0</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Rüdinger Spedition GmbH</t>
+          <t>Wiedmann &amp; Winz GmbH</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>https://www.spedition-ruedinger.de</t>
+          <t>https://www.wiedmann-winz.de</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>+49 6294 908-0</t>
+          <t>+49 7331 2000-0</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Wiedmann &amp; Winz GmbH</t>
+          <t>Alfred Schuon GmbH</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>https://www.wiedmann-winz.de</t>
+          <t>https://www.schuon.com</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>+49 7331 2000-0</t>
+          <t>+49 7456 693-0</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Alfred Schuon GmbH</t>
+          <t>L. Wackler Wwe. Nachf. GmbH, Spedition &amp; Logistik</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>https://www.schuon.com</t>
+          <t>https://www.wackler.de</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>+49 7456 693-0</t>
+          <t>+49 7161 806-0</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>L. Wackler Wwe. Nachf. GmbH, Spedition &amp; Logistik</t>
+          <t>Spedition Kübler GmbH</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>https://www.wackler.de</t>
+          <t>https://www.kuebler-spedition.de</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>+49 7161 806-0</t>
+          <t>+49 791 93000-0</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Spedition Kübler GmbH</t>
+          <t>Fritz GmbH &amp; Co. KG (Fritz Gruppe)</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>https://www.kuebler-spedition.de</t>
+          <t>https://www.fritz-gruppe.de</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>+49 791 93000-0</t>
+          <t>+49 7131 1573-0</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Fritz GmbH &amp; Co. KG (Fritz Gruppe)</t>
+          <t>Kleyling Spedition GmbH</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>https://www.fritz-gruppe.de</t>
+          <t>https://www.kleyling.de</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>+49 7131 1573-0</t>
+          <t>+49 7667 902-0</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Kleyling Spedition GmbH</t>
+          <t>Elflein Spedition &amp; Transport GmbH</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>https://www.kleyling.de</t>
+          <t>https://www.elflein.de</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>+49 7667 902-0</t>
+          <t>+49 951 96680-0</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Elflein Spedition &amp; Transport GmbH</t>
+          <t>Spedition Ansorge GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>https://www.elflein.de</t>
+          <t>https://www.ansorge-logistik.de</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>+49 951 96680-0</t>
+          <t>+49 8342 913-0</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Spedition Ansorge GmbH &amp; Co. KG</t>
+          <t>Ernst Frankenbach GmbH</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>https://www.ansorge-logistik.de</t>
+          <t>https://www.frankenbach.com</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>+49 8342 913-0</t>
+          <t>+49 6134 2900-100</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Ernst Frankenbach GmbH</t>
+          <t>Ludwig Meyer GmbH &amp; Co. KG (Meyer Logistik)</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>https://www.frankenbach.com</t>
+          <t>https://www.meyer-logistik.com</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>+49 6134 2900-100</t>
+          <t>+49 6175 4007-0</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Ludwig Meyer GmbH &amp; Co. KG (Meyer Logistik)</t>
+          <t>Meyer &amp; Meyer Holding SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>https://www.meyer-logistik.com</t>
+          <t>https://www.meyermeyer.com</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>+49 6175 4007-0</t>
+          <t>+49 541 9585-205</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Meyer &amp; Meyer Holding SE &amp; Co. KG</t>
+          <t>Streck Transportges. mbH</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>https://www.meyermeyer.com</t>
+          <t>https://www.streck-transport.com</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>+49 541 9585-205</t>
+          <t>+49 7621 177-0</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Streck Transportges. mbH</t>
+          <t>Vollers Group GmbH</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>https://www.streck-transport.com</t>
+          <t>https://www.vollers.com</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>+49 7621 177-0</t>
+          <t>+49 421 3892-00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Vollers Group GmbH</t>
+          <t>Wilhelm Rosebrock GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>https://www.vollers.com</t>
+          <t>https://www.rosebrock.com</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>+49 421 3892-00</t>
+          <t>+49 421 52000-0</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Wilhelm Rosebrock GmbH &amp; Co. KG</t>
+          <t>Kube &amp; Kubenz GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>https://www.rosebrock.com</t>
+          <t>https://www.kubekubenz.com</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>+49 421 52000-0</t>
+          <t>+49 40 237207-0</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Kube &amp; Kubenz GmbH &amp; Co. KG</t>
+          <t>Konrad Zippel Spediteur GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>https://www.kubekubenz.com</t>
+          <t>https://www.zippel24.com</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>+49 40 237207-0</t>
+          <t>+49 40 253045-0</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Konrad Zippel Spediteur GmbH &amp; Co. KG</t>
+          <t>KG Bursped Speditions-GmbH &amp; Co.</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>https://www.zippel24.com</t>
+          <t>https://www.bursped.de</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>+49 40 253045-0</t>
+          <t>+49 40 73123-0</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>KG Bursped Speditions-GmbH &amp; Co.</t>
+          <t>Winner Spedition GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>https://www.bursped.de</t>
+          <t>https://www.winner-spedition.de</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>+49 40 73123-0</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Winner Spedition GmbH &amp; Co. KG</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>https://www.winner-spedition.de</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
           <t>+49 2374 931-0</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C32"/>
+  <autoFilter ref="A1:C31"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -1028,7 +1011,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId31"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>